<commit_message>
#107 루아 enum 맵핑
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1,36 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\CSHYEON\Data\git\game\c++\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\cshyeon\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF825DCA-B7CE-49FA-9C09-3B266F89476A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE419CFC-4B4E-4522-B8E7-6E7C0C4309E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
     <sheet name="SEX" sheetId="1" r:id="rId1"/>
     <sheet name="DIRECTION" sheetId="2" r:id="rId2"/>
     <sheet name="DESTROY_TYPE" sheetId="18" r:id="rId3"/>
     <sheet name="OBJECT_TYPE" sheetId="3" r:id="rId4"/>
-    <sheet name="CREATURE" sheetId="4" r:id="rId5"/>
-    <sheet name="NATION" sheetId="5" r:id="rId6"/>
-    <sheet name="ACTION" sheetId="6" r:id="rId7"/>
-    <sheet name="STATE" sheetId="7" r:id="rId8"/>
-    <sheet name="CONDITION" sheetId="8" r:id="rId9"/>
-    <sheet name="SOUND" sheetId="9" r:id="rId10"/>
-    <sheet name="DURATION" sheetId="17" r:id="rId11"/>
-    <sheet name="STATE_LEVEL" sheetId="10" r:id="rId12"/>
-    <sheet name="CUSTOM_SETTING" sheetId="11" r:id="rId13"/>
-    <sheet name="MESSAGE_TYPE" sheetId="12" r:id="rId14"/>
-    <sheet name="SWAP_TYPE" sheetId="13" r:id="rId15"/>
-    <sheet name="CHAT_TYPE" sheetId="14" r:id="rId16"/>
-    <sheet name="WEATHER_TYPE" sheetId="15" r:id="rId17"/>
-    <sheet name="TIMER_TYPE" sheetId="16" r:id="rId18"/>
+    <sheet name="DIALOG_RESULT" sheetId="19" r:id="rId5"/>
+    <sheet name="CREATURE" sheetId="4" r:id="rId6"/>
+    <sheet name="NATION" sheetId="5" r:id="rId7"/>
+    <sheet name="ACTION" sheetId="6" r:id="rId8"/>
+    <sheet name="STATE" sheetId="7" r:id="rId9"/>
+    <sheet name="CONDITION" sheetId="8" r:id="rId10"/>
+    <sheet name="SOUND" sheetId="9" r:id="rId11"/>
+    <sheet name="DURATION" sheetId="17" r:id="rId12"/>
+    <sheet name="STATE_LEVEL" sheetId="10" r:id="rId13"/>
+    <sheet name="CUSTOM_SETTING" sheetId="11" r:id="rId14"/>
+    <sheet name="MESSAGE_TYPE" sheetId="12" r:id="rId15"/>
+    <sheet name="SWAP_TYPE" sheetId="13" r:id="rId16"/>
+    <sheet name="CHAT_TYPE" sheetId="14" r:id="rId17"/>
+    <sheet name="WEATHER_TYPE" sheetId="15" r:id="rId18"/>
+    <sheet name="TIMER_TYPE" sheetId="16" r:id="rId19"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="126">
   <si>
     <t>MAN</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -435,6 +436,18 @@
   </si>
   <si>
     <t>MOB | CHARACTER</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PREV</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QUIT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NEXT</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -875,6 +888,68 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DD5874E-E9B1-4690-9824-7FB4959F4820}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC28DC83-603A-4A95-BB7A-C0827113A5A5}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -937,7 +1012,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37600B40-33CE-4745-8CB9-BB2169DC8D7A}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1008,7 +1083,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE966F6D-82AF-41F8-894B-03F8136241A1}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1080,7 +1155,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD1ABC7A-1A46-42A2-B198-A73E04715834}">
   <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1192,7 +1267,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CDEFCDC-0D99-4CCA-AEFF-C483B2B7AA1B}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1270,7 +1345,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BB8BC29-7B8B-4407-82A2-F03CF66BF792}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -1297,7 +1372,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB782B33-B158-4B2E-A80C-B1B2C2B06F04}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -1340,7 +1415,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B212B2A-4A84-4835-BBA1-3FE883FFB899}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -1383,7 +1458,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{57336114-8A4F-4C9D-A254-6C6CDC1C1C51}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
@@ -1556,6 +1631,44 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C27EC380-0C98-4336-B006-077E82326FA2}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B1" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D30426EE-1EEF-4AE4-A8DB-5D3DB40D56EE}">
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1601,7 +1714,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1834AE54-D813-4ED8-8986-26E6279C1091}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1631,7 +1744,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{548D9DE6-D212-462C-9516-E80DD638149B}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1701,7 +1814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17FE56ED-F33B-47ED-86DC-276E9313D0F4}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
@@ -1769,66 +1882,4 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DD5874E-E9B1-4690-9824-7FB4959F4820}">
-  <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="16384" width="9" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add SLEEP action and update AFK timer
- Add SLEEP action to ACTION enum
- Update AFK timer to use SLEEP action instead of ATTACK
- Change idle threshold to 30 seconds in debug mode
- Update model files with new timestamp and formatting
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D58611-FF2D-4FB0-A356-B858A5088A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9951E1-FA90-4B59-B5AA-B640CCD88ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="5" activeTab="13" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="8" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
     <sheet name="SEX" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="138">
   <si>
     <t>MAN</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -500,6 +500,14 @@
   </si>
   <si>
     <t>ALL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SLEEP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EMOTION + 0x05</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2021,10 +2029,12 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{548D9DE6-D212-462C-9516-E80DD638149B}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="15.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -2083,6 +2093,14 @@
         <v>39</v>
       </c>
     </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor: rename sex to gender across codebase
- Rename SEX enum to GENDER in model and protocol
- Update character sex() method to gender() in C++ code
- Update FlatBuffer protocol definitions from sex to gender
- Update C# model and protocol classes from Sex to Gender
- Update database schema column from sex to gender
- Update DSL definitions from sex to gender
- Update Lua scripts to use gender instead of sex
- Update wiki submodule reference
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A9951E1-FA90-4B59-B5AA-B640CCD88ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDDAC12-6B0F-4977-811E-67A4846074C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="8" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
-    <sheet name="SEX" sheetId="1" r:id="rId1"/>
+    <sheet name="GENDER" sheetId="1" r:id="rId1"/>
     <sheet name="ROLE" sheetId="23" r:id="rId2"/>
     <sheet name="DIRECTION" sheetId="2" r:id="rId3"/>
     <sheet name="DESTROY_TYPE" sheetId="18" r:id="rId4"/>

</xml_diff>

<commit_message>
refactor: rename STATE enum and update cloaking visibility logic
- Rename STATE: TRANSLUCENCY to CLOACK, CLOACK to ADV_CLOACK
- Update enum.xlsx and generated model (C++/C#)
- Refactor character::state_to() for CLOACK/ADV_CLOACK visibility
- Fix detect() to pass true to update_external for cloaked characters
- Change 투명 spell to use STATE.CLOACK instead of HALF_CLOACK
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADDDAC12-6B0F-4977-811E-67A4846074C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564D9D05-A4A6-4CF9-85D4-B50A8069E1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
     <sheet name="GENDER" sheetId="1" r:id="rId1"/>
@@ -193,9 +193,6 @@
     <t>GHOST</t>
   </si>
   <si>
-    <t>TRANSLUCENCY</t>
-  </si>
-  <si>
     <t>RIDING</t>
   </si>
   <si>
@@ -205,309 +202,314 @@
     <t>HALF_CLOACK</t>
   </si>
   <si>
+    <t>NONE</t>
+  </si>
+  <si>
+    <t>HEAR</t>
+  </si>
+  <si>
+    <t>MAP</t>
+  </si>
+  <si>
+    <t>0x10</t>
+  </si>
+  <si>
+    <t>SWING</t>
+  </si>
+  <si>
+    <t>EQUIPMENT_OFF</t>
+  </si>
+  <si>
+    <t>EQUIPMENT_ON</t>
+  </si>
+  <si>
+    <t>DAMAGE</t>
+  </si>
+  <si>
+    <t>0x014B</t>
+  </si>
+  <si>
+    <t>0x0006</t>
+  </si>
+  <si>
+    <t>0x019A</t>
+  </si>
+  <si>
+    <t>0x019B</t>
+  </si>
+  <si>
+    <t>0x015D</t>
+  </si>
+  <si>
+    <t>SPELL</t>
+  </si>
+  <si>
+    <t>BASED</t>
+  </si>
+  <si>
+    <t>HP_MP</t>
+  </si>
+  <si>
+    <t>EXP_MONEY</t>
+  </si>
+  <si>
+    <t>0x40</t>
+  </si>
+  <si>
+    <t>0x20</t>
+  </si>
+  <si>
+    <t>WHISPER</t>
+  </si>
+  <si>
+    <t>GROUP</t>
+  </si>
+  <si>
+    <t>ROAR</t>
+  </si>
+  <si>
+    <t>ROAR_WORLDS</t>
+  </si>
+  <si>
+    <t>MAGIC_EFFECT</t>
+  </si>
+  <si>
+    <t>WEATHER_EFFECT</t>
+  </si>
+  <si>
+    <t>FIXED_MOVE</t>
+  </si>
+  <si>
+    <t>TRADE</t>
+  </si>
+  <si>
+    <t>FAST_MOVE</t>
+  </si>
+  <si>
+    <t>EFFECT_SOUND</t>
+  </si>
+  <si>
+    <t>NOTIFY</t>
+  </si>
+  <si>
+    <t>BLUE</t>
+  </si>
+  <si>
+    <t>STATE</t>
+  </si>
+  <si>
+    <t>SHOUT</t>
+  </si>
+  <si>
+    <t>WORLD</t>
+  </si>
+  <si>
+    <t>POPUP</t>
+  </si>
+  <si>
+    <t>YELLOW</t>
+  </si>
+  <si>
+    <t>BROWN</t>
+  </si>
+  <si>
+    <t>0x0C</t>
+  </si>
+  <si>
+    <t>ITEM</t>
+  </si>
+  <si>
+    <t>LIGHT_BLUE</t>
+  </si>
+  <si>
+    <t>RAIN</t>
+  </si>
+  <si>
+    <t>SNOW</t>
+  </si>
+  <si>
+    <t>BIRD</t>
+  </si>
+  <si>
+    <t>INCREASE</t>
+  </si>
+  <si>
+    <t>DECREASE</t>
+  </si>
+  <si>
+    <t>DISGUISE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x0019</t>
+  </si>
+  <si>
+    <t>FAST</t>
+  </si>
+  <si>
+    <t>THROW</t>
+  </si>
+  <si>
+    <t>0x0F</t>
+  </si>
+  <si>
+    <t>0x27</t>
+  </si>
+  <si>
+    <t>0x14</t>
+  </si>
+  <si>
+    <t>0x32</t>
+  </si>
+  <si>
+    <t>0x4E</t>
+  </si>
+  <si>
+    <t>0x28</t>
+  </si>
+  <si>
+    <t>DEFAULT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DEAD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CHARACTER</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MOB | CHARACTER</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PREV</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QUIT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NEXT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PK_PROTECT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x07</t>
+  </si>
+  <si>
+    <t>0x09</t>
+  </si>
+  <si>
+    <t>EXTENSION</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NONE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RED</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>YELLOW</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BLUE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x0D</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DIRECTION</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SIGHT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CHAT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BASED | HP_MP | EXP_MONEY | CROWD_CONTROL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CROWD_CONTROL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WEST</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EAST</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SOUTH</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NORTH</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WORLD</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GLOBAL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>USER</t>
+  </si>
+  <si>
+    <t>MODERATOR</t>
+  </si>
+  <si>
+    <t>ADMIN</t>
+  </si>
+  <si>
+    <t>SUPERADMIN</t>
+  </si>
+  <si>
+    <t>OWNER</t>
+  </si>
+  <si>
+    <t>MINIMUM</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ALL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SLEEP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>EMOTION + 0x05</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>CLOACK</t>
-  </si>
-  <si>
-    <t>NONE</t>
-  </si>
-  <si>
-    <t>HEAR</t>
-  </si>
-  <si>
-    <t>MAP</t>
-  </si>
-  <si>
-    <t>0x10</t>
-  </si>
-  <si>
-    <t>SWING</t>
-  </si>
-  <si>
-    <t>EQUIPMENT_OFF</t>
-  </si>
-  <si>
-    <t>EQUIPMENT_ON</t>
-  </si>
-  <si>
-    <t>DAMAGE</t>
-  </si>
-  <si>
-    <t>0x014B</t>
-  </si>
-  <si>
-    <t>0x0006</t>
-  </si>
-  <si>
-    <t>0x019A</t>
-  </si>
-  <si>
-    <t>0x019B</t>
-  </si>
-  <si>
-    <t>0x015D</t>
-  </si>
-  <si>
-    <t>SPELL</t>
-  </si>
-  <si>
-    <t>BASED</t>
-  </si>
-  <si>
-    <t>HP_MP</t>
-  </si>
-  <si>
-    <t>EXP_MONEY</t>
-  </si>
-  <si>
-    <t>0x40</t>
-  </si>
-  <si>
-    <t>0x20</t>
-  </si>
-  <si>
-    <t>WHISPER</t>
-  </si>
-  <si>
-    <t>GROUP</t>
-  </si>
-  <si>
-    <t>ROAR</t>
-  </si>
-  <si>
-    <t>ROAR_WORLDS</t>
-  </si>
-  <si>
-    <t>MAGIC_EFFECT</t>
-  </si>
-  <si>
-    <t>WEATHER_EFFECT</t>
-  </si>
-  <si>
-    <t>FIXED_MOVE</t>
-  </si>
-  <si>
-    <t>TRADE</t>
-  </si>
-  <si>
-    <t>FAST_MOVE</t>
-  </si>
-  <si>
-    <t>EFFECT_SOUND</t>
-  </si>
-  <si>
-    <t>NOTIFY</t>
-  </si>
-  <si>
-    <t>BLUE</t>
-  </si>
-  <si>
-    <t>STATE</t>
-  </si>
-  <si>
-    <t>SHOUT</t>
-  </si>
-  <si>
-    <t>WORLD</t>
-  </si>
-  <si>
-    <t>POPUP</t>
-  </si>
-  <si>
-    <t>YELLOW</t>
-  </si>
-  <si>
-    <t>BROWN</t>
-  </si>
-  <si>
-    <t>0x0C</t>
-  </si>
-  <si>
-    <t>ITEM</t>
-  </si>
-  <si>
-    <t>LIGHT_BLUE</t>
-  </si>
-  <si>
-    <t>RAIN</t>
-  </si>
-  <si>
-    <t>SNOW</t>
-  </si>
-  <si>
-    <t>BIRD</t>
-  </si>
-  <si>
-    <t>INCREASE</t>
-  </si>
-  <si>
-    <t>DECREASE</t>
-  </si>
-  <si>
-    <t>DISGUISE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0x0019</t>
-  </si>
-  <si>
-    <t>FAST</t>
-  </si>
-  <si>
-    <t>THROW</t>
-  </si>
-  <si>
-    <t>0x0F</t>
-  </si>
-  <si>
-    <t>0x27</t>
-  </si>
-  <si>
-    <t>0x14</t>
-  </si>
-  <si>
-    <t>0x32</t>
-  </si>
-  <si>
-    <t>0x4E</t>
-  </si>
-  <si>
-    <t>0x28</t>
-  </si>
-  <si>
-    <t>DEFAULT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DEAD</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CHARACTER</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>MOB | CHARACTER</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PREV</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>QUIT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NEXT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PK_PROTECT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0x07</t>
-  </si>
-  <si>
-    <t>0x09</t>
-  </si>
-  <si>
-    <t>EXTENSION</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NONE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>RED</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>YELLOW</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BLUE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>0x0D</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DIRECTION</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SIGHT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CHAT</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>BASED | HP_MP | EXP_MONEY | CROWD_CONTROL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CROWD_CONTROL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>WEST</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EAST</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SOUTH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>NORTH</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>WORLD</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>GLOBAL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>USER</t>
-  </si>
-  <si>
-    <t>MODERATOR</t>
-  </si>
-  <si>
-    <t>ADMIN</t>
-  </si>
-  <si>
-    <t>SUPERADMIN</t>
-  </si>
-  <si>
-    <t>OWNER</t>
-  </si>
-  <si>
-    <t>MINIMUM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ALL</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>SLEEP</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>EMOTION + 0x05</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ADV_CLOACK</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -944,7 +946,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="9" style="2"/>
+    <col min="1" max="1" width="13.875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
@@ -965,7 +968,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>136</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>24</v>
@@ -973,7 +976,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>25</v>
@@ -981,7 +984,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>36</v>
@@ -989,7 +992,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>37</v>
@@ -997,7 +1000,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>46</v>
+        <v>137</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>38</v>
@@ -1020,7 +1023,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
@@ -1028,7 +1031,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>23</v>
@@ -1036,7 +1039,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>24</v>
@@ -1044,7 +1047,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>36</v>
@@ -1052,7 +1055,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>39</v>
@@ -1060,10 +1063,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1083,10 +1086,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1094,39 +1097,39 @@
         <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1146,10 +1149,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -1157,7 +1160,7 @@
         <v>34</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -1165,7 +1168,7 @@
         <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1173,7 +1176,7 @@
         <v>31</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -1181,23 +1184,23 @@
         <v>30</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -1218,7 +1221,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>14</v>
@@ -1226,31 +1229,31 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>17</v>
@@ -1258,10 +1261,10 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1277,7 +1280,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -1285,7 +1288,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1293,7 +1296,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B3">
         <v>3</v>
@@ -1301,7 +1304,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -1320,7 +1323,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -1328,7 +1331,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1352,7 +1355,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
@@ -1360,7 +1363,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>23</v>
@@ -1368,7 +1371,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>24</v>
@@ -1376,7 +1379,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>25</v>
@@ -1384,7 +1387,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>36</v>
@@ -1392,7 +1395,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>37</v>
@@ -1400,7 +1403,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>38</v>
@@ -1408,15 +1411,15 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>39</v>
@@ -1424,15 +1427,15 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>35</v>
@@ -1440,10 +1443,10 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1462,7 +1465,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
@@ -1470,7 +1473,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>23</v>
@@ -1478,7 +1481,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>25</v>
@@ -1486,7 +1489,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>36</v>
@@ -1494,7 +1497,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>37</v>
@@ -1502,7 +1505,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>39</v>
@@ -1510,7 +1513,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>35</v>
@@ -1518,10 +1521,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>
@@ -1537,7 +1540,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B1" t="s">
         <v>22</v>
@@ -1545,7 +1548,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
@@ -1568,7 +1571,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -1576,7 +1579,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1584,7 +1587,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -1592,7 +1595,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -1600,7 +1603,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
@@ -1627,7 +1630,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
@@ -1635,7 +1638,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
         <v>24</v>
@@ -1643,7 +1646,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
@@ -1670,7 +1673,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
@@ -1678,7 +1681,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
         <v>24</v>
@@ -1686,7 +1689,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B4" t="s">
         <v>25</v>
@@ -1705,7 +1708,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B1" t="s">
         <v>23</v>
@@ -1713,7 +1716,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
         <v>24</v>
@@ -1732,7 +1735,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -1740,7 +1743,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1748,7 +1751,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1756,7 +1759,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -1821,7 +1824,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -1829,7 +1832,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1885,7 +1888,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>17</v>
@@ -1896,7 +1899,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
@@ -1923,7 +1926,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -1931,7 +1934,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1939,7 +1942,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -2095,10 +2098,10 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: align object type flags and quest cleanup
- Update OBJECT_TYPE enum bit flags in data table and regenerated model files
- Fix object type membership check logic in object::is using ENUM_IN
- Clear related achievement when king quest curse branch is executed
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564D9D05-A4A6-4CF9-85D4-B50A8069E1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28434FB-25FC-49B4-B7A4-1DC6FBE1CB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="9" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
     <sheet name="GENDER" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="139">
   <si>
     <t>MAN</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -97,10 +97,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ITEM | NPC | MOB</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>0x01</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -109,82 +105,74 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>0x08</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PHOENIX</t>
+  </si>
+  <si>
+    <t>TIGER</t>
+  </si>
+  <si>
+    <t>TURTLE</t>
+  </si>
+  <si>
+    <t>DRAGON</t>
+  </si>
+  <si>
+    <t>0x00</t>
+  </si>
+  <si>
+    <t>0x01</t>
+  </si>
+  <si>
     <t>0x02</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x03</t>
+  </si>
+  <si>
+    <t>GOGURYEO</t>
+  </si>
+  <si>
+    <t>BUYEO</t>
+  </si>
+  <si>
+    <t>ATTACK</t>
+  </si>
+  <si>
+    <t>ARROW</t>
+  </si>
+  <si>
+    <t>EMOTION</t>
+  </si>
+  <si>
+    <t>PICKUP</t>
+  </si>
+  <si>
+    <t>PICKUP_SILENT</t>
+  </si>
+  <si>
+    <t>CAST_SPELL</t>
+  </si>
+  <si>
+    <t>EAT</t>
+  </si>
+  <si>
+    <t>0x0B</t>
   </si>
   <si>
     <t>0x04</t>
-    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x05</t>
+  </si>
+  <si>
+    <t>0x06</t>
   </si>
   <si>
     <t>0x08</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>PHOENIX</t>
-  </si>
-  <si>
-    <t>TIGER</t>
-  </si>
-  <si>
-    <t>TURTLE</t>
-  </si>
-  <si>
-    <t>DRAGON</t>
-  </si>
-  <si>
-    <t>0x00</t>
-  </si>
-  <si>
-    <t>0x01</t>
-  </si>
-  <si>
-    <t>0x02</t>
-  </si>
-  <si>
-    <t>0x03</t>
-  </si>
-  <si>
-    <t>GOGURYEO</t>
-  </si>
-  <si>
-    <t>BUYEO</t>
-  </si>
-  <si>
-    <t>ATTACK</t>
-  </si>
-  <si>
-    <t>ARROW</t>
-  </si>
-  <si>
-    <t>EMOTION</t>
-  </si>
-  <si>
-    <t>PICKUP</t>
-  </si>
-  <si>
-    <t>PICKUP_SILENT</t>
-  </si>
-  <si>
-    <t>CAST_SPELL</t>
-  </si>
-  <si>
-    <t>EAT</t>
-  </si>
-  <si>
-    <t>0x0B</t>
-  </si>
-  <si>
-    <t>0x04</t>
-  </si>
-  <si>
-    <t>0x05</t>
-  </si>
-  <si>
-    <t>0x06</t>
-  </si>
-  <si>
-    <t>0x08</t>
   </si>
   <si>
     <t>NORMAL</t>
@@ -380,10 +368,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MOB | CHARACTER</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>PREV</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -510,6 +494,26 @@
   </si>
   <si>
     <t>ADV_CLOACK</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x02 | OBJECT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x100 | OBJECT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x200 | OBJECT</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x400 | LIFE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0x800 | LIFE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -952,58 +956,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1023,50 +1027,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1086,50 +1090,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1149,58 +1153,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>92</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1221,50 +1225,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>59</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>60</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
   </sheetData>
@@ -1280,7 +1284,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -1288,7 +1292,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1296,7 +1300,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B3">
         <v>3</v>
@@ -1304,7 +1308,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -1323,7 +1327,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -1331,7 +1335,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1355,98 +1359,98 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1465,66 +1469,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1540,18 +1544,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1571,7 +1575,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -1579,7 +1583,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1587,7 +1591,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -1595,7 +1599,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -1603,7 +1607,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
@@ -1622,34 +1626,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1665,34 +1669,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -1708,18 +1712,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -1735,7 +1739,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -1743,7 +1747,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1751,7 +1755,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1759,7 +1763,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -1824,7 +1828,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -1832,7 +1836,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1859,55 +1863,55 @@
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>15</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>102</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>17</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>103</v>
+        <v>137</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>99</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -1926,7 +1930,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -1934,7 +1938,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1942,7 +1946,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -1964,34 +1968,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -2010,18 +2014,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -2042,66 +2046,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: rename GENDER enum to MALE and FEMALE
- Update enum.xlsx, item.xlsx, and regenerated model.h
- Apply renames in C++ game server, bot, and tests
- Sync HTTP Model.cs and Lua scripts with new GENDER values
- Use const reference when iterating spawned_mobs in stat.cpp
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A28434FB-25FC-49B4-B7A4-1DC6FBE1CB86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17523AF0-224C-4364-822B-AD6506D964C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
     <sheet name="GENDER" sheetId="1" r:id="rId1"/>
@@ -49,14 +49,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="139">
   <si>
-    <t>MAN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>WOMAN</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>LEFT</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -514,6 +506,14 @@
   </si>
   <si>
     <t>0x800 | LIFE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MALE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FEMALE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -925,7 +925,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>137</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -933,7 +933,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>138</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -956,58 +956,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1027,50 +1027,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1090,50 +1090,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1153,58 +1153,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>91</v>
-      </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1225,50 +1225,50 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1284,7 +1284,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -1292,7 +1292,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1300,7 +1300,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B3">
         <v>3</v>
@@ -1308,7 +1308,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B4">
         <v>4</v>
@@ -1327,7 +1327,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B1">
         <v>1</v>
@@ -1335,7 +1335,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B2">
         <v>2</v>
@@ -1359,98 +1359,98 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1469,66 +1469,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1544,18 +1544,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1575,7 +1575,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -1583,7 +1583,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1591,7 +1591,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -1599,7 +1599,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -1607,7 +1607,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
@@ -1626,34 +1626,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1669,34 +1669,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1712,18 +1712,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1739,7 +1739,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -1747,7 +1747,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1755,7 +1755,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B3">
         <v>2</v>
@@ -1763,7 +1763,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -1785,7 +1785,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1801,7 +1801,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -1809,7 +1809,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
@@ -1828,7 +1828,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B1">
         <v>0</v>
@@ -1836,7 +1836,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -1860,58 +1860,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1930,7 +1930,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B1" s="1">
         <v>0</v>
@@ -1938,7 +1938,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
@@ -1946,7 +1946,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
@@ -1968,34 +1968,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2014,18 +2014,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -2046,66 +2046,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add instance_rule entry routing
- Route map entry by CAPACITY and GROUP instance rules
- Copy instance tiles from source map instead of reloading assets
- Track character_count on base map for capacity checks
- Force group leave/kick/destroy back to source with skip_instance_rule
- Keep /맵이동 on S unless an explicit slot is given
- Add instance_rule and instance_capacity model fields and Lua builtins
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17523AF0-224C-4364-822B-AD6506D964C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F74BA1-27C1-4D0F-AC79-06DDDA867163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" firstSheet="14" activeTab="23" xr2:uid="{08B6B988-6A34-4205-94C2-FA55368096A2}"/>
   </bookViews>
   <sheets>
     <sheet name="GENDER" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,7 @@
     <sheet name="WEATHER_TYPE" sheetId="15" r:id="rId21"/>
     <sheet name="TIMER_TYPE" sheetId="16" r:id="rId22"/>
     <sheet name="HEAD_MARKER" sheetId="20" r:id="rId23"/>
+    <sheet name="INSTANCE_RULE_TYPE" sheetId="24" r:id="rId24"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="141">
   <si>
     <t>LEFT</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -514,6 +515,14 @@
   </si>
   <si>
     <t>FEMALE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CAPACITY</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>GROUP</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1775,6 +1784,44 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{06B9EE36-D448-4820-A80D-20F18C0D7C67}">
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="16384" width="9" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEFB188D-3B26-41D9-B64A-51D7BDB1D0A9}">
   <dimension ref="A1:B4"/>

</xml_diff>

<commit_message>
feat: add delirious chat scramble and dialog QUIT/TOP handling
- Add assert_korean completed mode, is_ksx1001_hangul, and delirious scramble
- Apply delirious on life chat; wire poison spell 3059 buff hooks
- Standardize dialog scripts: QUIT exits first, TOP goes to parent, drop nil guards
- Fix CP949 assert_korean call sites in login and bot
- Update related dialog/click builtins and generated model enums
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1985,53 +1985,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
-  <cols>
-    <col width="9" customWidth="1" style="1" min="1" max="16384"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>PREV</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>QUIT</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>NEXT</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>2</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
@@ -2041,6 +1994,63 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>PREV</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>QUIT</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>NEXT</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>TOP</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
+  <cols>
+    <col width="9" customWidth="1" style="1" min="1" max="16384"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>PHOENIX</t>
         </is>
       </c>
@@ -2138,7 +2148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="1"/>
@@ -2243,28 +2253,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="0" t="inlineStr">
         <is>
           <t>SLEEP</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="0" t="inlineStr">
         <is>
           <t>EMOTION + 0x05</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: migrate menus to pursuit and extend bot wait-only request
- Switch NPC dialog menus from list to pursuit (0x2F)
- Update dialog bot helpers and related integration tests
- Allow nil packet on bot request/request_on for wait-only hooks
- Expand poison skill test for tick damage, delirious chat, and HP floor
- Align click TOP handling and related script/model updates
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1985,7 +1985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="9" customWidth="1" style="1" min="1" max="16384"/>
@@ -2019,16 +2019,6 @@
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>TOP</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: persist hair, face, helmet option, and appearance
- Rename user look to hair and store face, reputation, and evaluation
- Add visible helmet option and fill v651 appearance from equipment
- Update login, HTTP, and group portrait paths
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1134,7 +1134,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="15.25" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -1293,6 +1293,18 @@
         </is>
       </c>
       <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>0x0E</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>VISIBLE_HELMET</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
         <is>
           <t>0x0E</t>
         </is>

</xml_diff>

<commit_message>
feat: add TIMER_TYPE.OFF and pass enum to timer
- Add TIMER_TYPE.OFF to enum table and generated models
- Change character, map, and server timer builtins to take TIMER_TYPE
- Update Lua callers and /타이머 to use TIMER_TYPE
</commit_message>
<xml_diff>
--- a/resources/table/enum.xlsx
+++ b/resources/table/enum.xlsx
@@ -1664,7 +1664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <sheetData>
     <row r="1">
@@ -1688,6 +1688,18 @@
       <c r="B2" s="0" t="inlineStr">
         <is>
           <t>0x02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>OFF</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x03</t>
         </is>
       </c>
     </row>

</xml_diff>